<commit_message>
Update task files and add results
</commit_message>
<xml_diff>
--- a/debug/excel_overviews/overview_aae.xlsx
+++ b/debug/excel_overviews/overview_aae.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="239">
   <si>
     <t>vs_Llama-2-7b-chat-hf</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>vs_gemini-1.5-flash</t>
+  </si>
+  <si>
+    <t>vs_gpt-4.1_errors</t>
   </si>
   <si>
     <t>Judge Model</t>
@@ -260,6 +263,34 @@
 V1: 95 V2: 33 Vties: 14</t>
   </si>
   <si>
+    <t>ASR: 0.65
+V1: 107 V2: 2 Vties: 33</t>
+  </si>
+  <si>
+    <t>ASR: 0.83
+V1: 103 V2: 11 Vties: 24</t>
+  </si>
+  <si>
+    <t>ASR: 0.82
+V1: 125 V2: 8 Vties: 9</t>
+  </si>
+  <si>
+    <t>ASR: 0.74
+V1: 136 V2: 1 Vties: 5</t>
+  </si>
+  <si>
+    <t>ASR: 0.83
+V1: 101 V2: 1 Vties: 40</t>
+  </si>
+  <si>
+    <t>ASR: 0.85
+V1: 61 V2: 26 Vties: 54</t>
+  </si>
+  <si>
+    <t>ASR: 0.85
+V1: 130 V2: 2 Vties: 10</t>
+  </si>
+  <si>
     <t>AASR: 0.00
 V1: 123 V2: 7 Vties: 12</t>
   </si>
@@ -452,6 +483,34 @@
 V1: 95 V2: 33 Vties: 14</t>
   </si>
   <si>
+    <t>AASR: 0.00
+V1: 107 V2: 2 Vties: 33</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 103 V2: 11 Vties: 24</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 125 V2: 8 Vties: 9</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 136 V2: 1 Vties: 5</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 101 V2: 1 Vties: 40</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 61 V2: 26 Vties: 54</t>
+  </si>
+  <si>
+    <t>AASR: 0.00
+V1: 130 V2: 2 Vties: 10</t>
+  </si>
+  <si>
     <t>FR: 0.68
 V1: 123 V2: 7 Vties: 12</t>
   </si>
@@ -648,6 +707,34 @@
 V1: 95 V2: 33 Vties: 14</t>
   </si>
   <si>
+    <t>FR: 0.73
+V1: 107 V2: 2 Vties: 33</t>
+  </si>
+  <si>
+    <t>FR: 0.80
+V1: 103 V2: 11 Vties: 24</t>
+  </si>
+  <si>
+    <t>FR: 0.78
+V1: 125 V2: 8 Vties: 9</t>
+  </si>
+  <si>
+    <t>FR: 0.74
+V1: 136 V2: 1 Vties: 5</t>
+  </si>
+  <si>
+    <t>FR: 0.87
+V1: 101 V2: 1 Vties: 40</t>
+  </si>
+  <si>
+    <t>FR: 0.75
+V1: 61 V2: 26 Vties: 54</t>
+  </si>
+  <si>
+    <t>FR: 0.85
+V1: 130 V2: 2 Vties: 10</t>
+  </si>
+  <si>
     <t>CR: 0.35
 V1: 123 V2: 7 Vties: 12</t>
   </si>
@@ -842,6 +929,34 @@
   <si>
     <t>CR: 0.27
 V1: 95 V2: 33 Vties: 14</t>
+  </si>
+  <si>
+    <t>CR: 0.36
+V1: 107 V2: 2 Vties: 33</t>
+  </si>
+  <si>
+    <t>CR: 0.25
+V1: 103 V2: 11 Vties: 24</t>
+  </si>
+  <si>
+    <t>CR: 0.23
+V1: 125 V2: 8 Vties: 9</t>
+  </si>
+  <si>
+    <t>CR: 0.27
+V1: 136 V2: 1 Vties: 5</t>
+  </si>
+  <si>
+    <t>CR: 0.18
+V1: 101 V2: 1 Vties: 40</t>
+  </si>
+  <si>
+    <t>CR: 0.40
+V1: 61 V2: 26 Vties: 54</t>
+  </si>
+  <si>
+    <t>CR: 0.16
+V1: 130 V2: 2 Vties: 10</t>
   </si>
 </sst>
 </file>
@@ -1202,15 +1317,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="20.7109375" style="1" customWidth="1"/>
+    <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1233,187 +1348,211 @@
       <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1423,15 +1562,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="20.7109375" style="1" customWidth="1"/>
+    <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1454,187 +1593,211 @@
       <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="C8" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="G8" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1644,15 +1807,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="20.7109375" style="1" customWidth="1"/>
+    <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1675,187 +1838,211 @@
       <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>139</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>160</v>
+        <v>175</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -1865,15 +2052,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="20.7109375" style="1" customWidth="1"/>
+    <col min="1" max="10" width="20.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1896,187 +2083,211 @@
       <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>209</v>
+        <v>231</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>